<commit_message>
Remove old tech diagnostics text from translations data
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -1460,11 +1460,7 @@
           <t>hero_desc</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>With over 8 years in tech diagnostics, I solve and learn complex problems and i am currently exploring the world of open-source softwares,  2d games  development via a.i. tools.</t>
-        </is>
-      </c>
+      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>আমি মো. মুকিদ হাসান সিয়াম। টেক ডায়াগনস্টিক্সে ৮ বছরেরও বেশি সময় ধরে জটিল সমস্যার সমাধান করছি এবং বর্তমানে ওপেন-সোর্স গেম ডেভেলপমেন্টের জগৎ নিয়ে কাজ করছি।</t>

</xml_diff>